<commit_message>
Added docs/session/site-load-report-under-and-over-nameplate.txt and updated docs/session/Rough_kW_kVA_Table.xlsx with over nameplate info.
</commit_message>
<xml_diff>
--- a/docs/session/Rough_kW_kVA_Table.xlsx
+++ b/docs/session/Rough_kW_kVA_Table.xlsx
@@ -11,13 +11,13 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="BREAKER_RATING_A" vbProcedure="false">Sheet1!$B$17</definedName>
-    <definedName function="false" hidden="false" name="CONTINUOUS_DUTY_DERATE" vbProcedure="false">Sheet1!$B$18</definedName>
-    <definedName function="false" hidden="false" name="ev_apparent_power_kva" vbProcedure="false">Sheet1!$B$21</definedName>
-    <definedName function="false" hidden="false" name="ev_pilot_current_a" vbProcedure="false">Sheet1!$B$20</definedName>
-    <definedName function="false" hidden="false" name="ev_real_power_kw" vbProcedure="false">Sheet1!$B$22</definedName>
-    <definedName function="false" hidden="false" name="EV_TRUE_POWER_FACTOR" vbProcedure="false">Sheet1!$B$19</definedName>
-    <definedName function="false" hidden="false" name="PANEL_VOLTAGE_V" vbProcedure="false">Sheet1!$B$16</definedName>
+    <definedName function="false" hidden="false" name="BREAKER_RATING_A" vbProcedure="false">Sheet1!$B$23</definedName>
+    <definedName function="false" hidden="false" name="CONTINUOUS_DUTY_DERATE" vbProcedure="false">Sheet1!$B$24</definedName>
+    <definedName function="false" hidden="false" name="ev_apparent_power_kva" vbProcedure="false">Sheet1!$B$27</definedName>
+    <definedName function="false" hidden="false" name="ev_pilot_current_a" vbProcedure="false">Sheet1!$B$26</definedName>
+    <definedName function="false" hidden="false" name="ev_real_power_kw" vbProcedure="false">Sheet1!$B$28</definedName>
+    <definedName function="false" hidden="false" name="EV_TRUE_POWER_FACTOR" vbProcedure="false">Sheet1!$B$25</definedName>
+    <definedName function="false" hidden="false" name="PANEL_VOLTAGE_V" vbProcedure="false">Sheet1!$B$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="20">
   <si>
     <t xml:space="preserve">ROUGH KW AND KVA APPROXIMATIONS VS. EXACT NUMBERS</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">PF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">over nameplate -&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">PANEL_VOLTAGE_V</t>
@@ -181,7 +184,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -206,6 +209,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -223,8 +230,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R28"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="1.68"/>
@@ -854,61 +861,347 @@
         <v>-0.0015326450487132</v>
       </c>
     </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="O15" s="5"/>
+    </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="B16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="C16" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="1" t="n">
+        <f aca="false">$B$5 *C16</f>
+        <v>73.326</v>
+      </c>
+      <c r="F16" s="1" t="n">
+        <f aca="false">E16/$B$6</f>
+        <v>74.8224489795918</v>
+      </c>
+      <c r="G16" s="1" t="n">
+        <f aca="false">E16/$C16</f>
+        <v>6.666</v>
+      </c>
+      <c r="H16" s="1" t="n">
+        <f aca="false">F16/$C16</f>
+        <v>6.80204081632653</v>
+      </c>
+      <c r="I16" s="5"/>
+      <c r="J16" s="1" t="n">
+        <v>74.36</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>75.76</v>
+      </c>
+      <c r="L16" s="1" t="n">
+        <f aca="false">J16/$C16</f>
+        <v>6.76</v>
+      </c>
+      <c r="M16" s="1" t="n">
+        <f aca="false">K16/$C16</f>
+        <v>6.88727272727273</v>
+      </c>
+      <c r="N16" s="1" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="O16" s="5"/>
+      <c r="P16" s="1" t="n">
+        <f aca="false">G16 - L16</f>
+        <v>-0.0939999999999994</v>
+      </c>
+      <c r="Q16" s="1" t="n">
+        <f aca="false">H16 - M16</f>
+        <v>-0.085231910946197</v>
+      </c>
+      <c r="R16" s="1" t="n">
+        <f aca="false">$B$6 - N16</f>
+        <v>-0.001</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="1" t="n">
+        <f aca="false">$B$5 *C17</f>
+        <v>99.99</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <f aca="false">E17/$B$6</f>
+        <v>102.030612244898</v>
+      </c>
+      <c r="G17" s="1" t="n">
+        <f aca="false">E17/$C17</f>
+        <v>6.666</v>
+      </c>
+      <c r="H17" s="1" t="n">
+        <f aca="false">F17/$C17</f>
+        <v>6.80204081632653</v>
+      </c>
+      <c r="I17" s="5"/>
+      <c r="J17" s="1" t="n">
+        <v>102.03</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="L17" s="1" t="n">
+        <f aca="false">J17/$C17</f>
+        <v>6.802</v>
+      </c>
+      <c r="M17" s="1" t="n">
+        <f aca="false">K17/$C17</f>
+        <v>6.94</v>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="O17" s="5"/>
+      <c r="P17" s="1" t="n">
+        <f aca="false">G17 - L17</f>
+        <v>-0.136</v>
+      </c>
+      <c r="Q17" s="1" t="n">
+        <f aca="false">H17 - M17</f>
+        <v>-0.137959183673469</v>
+      </c>
+      <c r="R17" s="1" t="n">
+        <f aca="false">$B$6 - N17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="1" t="n">
+        <f aca="false">$B$5 *C18</f>
+        <v>133.32</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <f aca="false">E18/$B$6</f>
+        <v>136.040816326531</v>
+      </c>
+      <c r="G18" s="1" t="n">
+        <f aca="false">E18/$C18</f>
+        <v>6.666</v>
+      </c>
+      <c r="H18" s="1" t="n">
+        <f aca="false">F18/$C18</f>
+        <v>6.80204081632653</v>
+      </c>
+      <c r="I18" s="5"/>
+      <c r="J18" s="1" t="n">
+        <v>137.18</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>140.29</v>
+      </c>
+      <c r="L18" s="1" t="n">
+        <f aca="false">J18/$C18</f>
+        <v>6.859</v>
+      </c>
+      <c r="M18" s="1" t="n">
+        <f aca="false">K18/$C18</f>
+        <v>7.0145</v>
+      </c>
+      <c r="N18" s="1" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="O18" s="5"/>
+      <c r="P18" s="1" t="n">
+        <f aca="false">G18 - L18</f>
+        <v>-0.193000000000001</v>
+      </c>
+      <c r="Q18" s="1" t="n">
+        <f aca="false">H18 - M18</f>
+        <v>-0.21245918367347</v>
+      </c>
+      <c r="R18" s="1" t="n">
+        <f aca="false">$B$6 - N18</f>
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="1" t="n">
+        <f aca="false">$B$5 *C19</f>
+        <v>199.98</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <f aca="false">E19/$B$6</f>
+        <v>204.061224489796</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <f aca="false">E19/$C19</f>
+        <v>6.666</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <f aca="false">F19/$C19</f>
+        <v>6.80204081632653</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="1" t="n">
+        <v>209.37</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>215.33</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <f aca="false">J19/$C19</f>
+        <v>6.979</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <f aca="false">K19/$C19</f>
+        <v>7.17766666666667</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="O19" s="5"/>
+      <c r="P19" s="1" t="n">
+        <f aca="false">G19 - L19</f>
+        <v>-0.313</v>
+      </c>
+      <c r="Q19" s="1" t="n">
+        <f aca="false">H19 - M19</f>
+        <v>-0.375625850340136</v>
+      </c>
+      <c r="R19" s="1" t="n">
+        <f aca="false">$B$6 - N19</f>
+        <v>0.00800000000000001</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="1" t="n">
+        <f aca="false">$B$5 *C20</f>
+        <v>333.3</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <f aca="false">E20/$B$6</f>
+        <v>340.102040816327</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <f aca="false">E20/$C20</f>
+        <v>6.666</v>
+      </c>
+      <c r="H20" s="1" t="n">
+        <f aca="false">F20/$C20</f>
+        <v>6.80204081632653</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="1" t="n">
+        <v>361.33</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>376.59</v>
+      </c>
+      <c r="L20" s="1" t="n">
+        <f aca="false">J20/$C20</f>
+        <v>7.2266</v>
+      </c>
+      <c r="M20" s="1" t="n">
+        <f aca="false">K20/$C20</f>
+        <v>7.5318</v>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="O20" s="5"/>
+      <c r="P20" s="1" t="n">
+        <f aca="false">G20 - L20</f>
+        <v>-0.560599999999999</v>
+      </c>
+      <c r="Q20" s="1" t="n">
+        <f aca="false">H20 - M20</f>
+        <v>-0.729759183673468</v>
+      </c>
+      <c r="R20" s="1" t="n">
+        <f aca="false">$B$6 - N20</f>
+        <v>0.021</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="0" t="n">
         <v>208</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="0" t="n">
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" s="0" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="0" t="n">
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="0" t="n">
         <v>0.8</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="0" t="n">
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="0" t="n">
         <v>0.99</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="0" t="n">
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="0" t="n">
         <f aca="false">BREAKER_RATING_A * CONTINUOUS_DUTY_DERATE</f>
         <v>32</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21" s="0" t="n">
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="0" t="n">
         <f aca="false">PANEL_VOLTAGE_V * ev_pilot_current_a / 1000</f>
         <v>6.656</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="0" t="n">
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="0" t="n">
         <f aca="false">ev_apparent_power_kva * EV_TRUE_POWER_FACTOR</f>
         <v>6.58944</v>
       </c>

</xml_diff>

<commit_message>
Updated docs/session/Rough_kW_kVA_Table.xlsx and archived 3 other docs.
</commit_message>
<xml_diff>
--- a/docs/session/Rough_kW_kVA_Table.xlsx
+++ b/docs/session/Rough_kW_kVA_Table.xlsx
@@ -11,13 +11,13 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="BREAKER_RATING_A" vbProcedure="false">Sheet1!$B$23</definedName>
-    <definedName function="false" hidden="false" name="CONTINUOUS_DUTY_DERATE" vbProcedure="false">Sheet1!$B$24</definedName>
-    <definedName function="false" hidden="false" name="ev_apparent_power_kva" vbProcedure="false">Sheet1!$B$27</definedName>
-    <definedName function="false" hidden="false" name="ev_pilot_current_a" vbProcedure="false">Sheet1!$B$26</definedName>
-    <definedName function="false" hidden="false" name="ev_real_power_kw" vbProcedure="false">Sheet1!$B$28</definedName>
-    <definedName function="false" hidden="false" name="EV_TRUE_POWER_FACTOR" vbProcedure="false">Sheet1!$B$25</definedName>
-    <definedName function="false" hidden="false" name="PANEL_VOLTAGE_V" vbProcedure="false">Sheet1!$B$22</definedName>
+    <definedName function="false" hidden="false" name="BREAKER_RATING_A" vbProcedure="false">Sheet1!$B$17</definedName>
+    <definedName function="false" hidden="false" name="CONTINUOUS_DUTY_DERATE" vbProcedure="false">Sheet1!$B$18</definedName>
+    <definedName function="false" hidden="false" name="ev_apparent_power_kva" vbProcedure="false">Sheet1!$B$21</definedName>
+    <definedName function="false" hidden="false" name="ev_pilot_current_a" vbProcedure="false">Sheet1!$B$20</definedName>
+    <definedName function="false" hidden="false" name="ev_real_power_kw" vbProcedure="false">Sheet1!$B$22</definedName>
+    <definedName function="false" hidden="false" name="EV_TRUE_POWER_FACTOR" vbProcedure="false">Sheet1!$B$19</definedName>
+    <definedName function="false" hidden="false" name="PANEL_VOLTAGE_V" vbProcedure="false">Sheet1!$B$16</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t xml:space="preserve">ROUGH KW AND KVA APPROXIMATIONS VS. EXACT NUMBERS</t>
   </si>
@@ -65,9 +65,6 @@
   </si>
   <si>
     <t xml:space="preserve">PF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">over nameplate -&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">PANEL_VOLTAGE_V</t>
@@ -184,7 +181,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -209,10 +206,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -230,8 +223,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:R22"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="1.68"/>
@@ -338,35 +331,35 @@
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="1" t="n">
-        <v>6.95</v>
+        <v>6.8</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>7.37</v>
+        <v>7.22</v>
       </c>
       <c r="L5" s="1" t="n">
         <f aca="false">J5/$C5</f>
-        <v>6.95</v>
+        <v>6.8</v>
       </c>
       <c r="M5" s="1" t="n">
         <f aca="false">K5/$C5</f>
-        <v>7.37</v>
+        <v>7.22</v>
       </c>
       <c r="N5" s="1" t="n">
         <f aca="false">J5 / K5</f>
-        <v>0.943012211668928</v>
+        <v>0.941828254847645</v>
       </c>
       <c r="O5" s="5"/>
       <c r="P5" s="1" t="n">
         <f aca="false">G5 - L5</f>
-        <v>-0.284</v>
+        <v>-0.133999999999999</v>
       </c>
       <c r="Q5" s="1" t="n">
         <f aca="false">H5 - M5</f>
-        <v>-0.567959183673469</v>
+        <v>-0.41795918367347</v>
       </c>
       <c r="R5" s="1" t="n">
         <f aca="false">$B$6 - N5</f>
-        <v>0.0369877883310719</v>
+        <v>0.0381717451523546</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -398,35 +391,35 @@
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="1" t="n">
-        <v>13.58</v>
+        <v>13.42</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>14.01</v>
+        <v>13.85</v>
       </c>
       <c r="L6" s="1" t="n">
         <f aca="false">J6/$C6</f>
-        <v>6.79</v>
+        <v>6.71</v>
       </c>
       <c r="M6" s="1" t="n">
         <f aca="false">K6/$C6</f>
-        <v>7.005</v>
+        <v>6.925</v>
       </c>
       <c r="N6" s="1" t="n">
         <f aca="false">J6 / K6</f>
-        <v>0.969307637401856</v>
+        <v>0.968953068592058</v>
       </c>
       <c r="O6" s="5"/>
       <c r="P6" s="1" t="n">
         <f aca="false">G6 - L6</f>
-        <v>-0.124</v>
+        <v>-0.0439999999999996</v>
       </c>
       <c r="Q6" s="1" t="n">
         <f aca="false">H6 - M6</f>
-        <v>-0.202959183673469</v>
+        <v>-0.12295918367347</v>
       </c>
       <c r="R6" s="1" t="n">
         <f aca="false">$B$6 - N6</f>
-        <v>0.0106923625981441</v>
+        <v>0.0110469314079422</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -452,35 +445,35 @@
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="1" t="n">
-        <v>20.23</v>
+        <v>20.06</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>20.72</v>
+        <v>20.55</v>
       </c>
       <c r="L7" s="1" t="n">
         <f aca="false">J7/$C7</f>
-        <v>6.74333333333333</v>
+        <v>6.68666666666667</v>
       </c>
       <c r="M7" s="1" t="n">
         <f aca="false">K7/$C7</f>
-        <v>6.90666666666667</v>
+        <v>6.85</v>
       </c>
       <c r="N7" s="1" t="n">
         <f aca="false">J7 / K7</f>
-        <v>0.976351351351351</v>
+        <v>0.976155717761557</v>
       </c>
       <c r="O7" s="5"/>
       <c r="P7" s="1" t="n">
         <f aca="false">G7 - L7</f>
-        <v>-0.0773333333333328</v>
+        <v>-0.0206666666666662</v>
       </c>
       <c r="Q7" s="1" t="n">
         <f aca="false">H7 - M7</f>
-        <v>-0.104625850340135</v>
+        <v>-0.0479591836734707</v>
       </c>
       <c r="R7" s="1" t="n">
         <f aca="false">$B$6 - N7</f>
-        <v>0.00364864864864856</v>
+        <v>0.00384428223844291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -506,35 +499,35 @@
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="1" t="n">
-        <v>26.91</v>
+        <v>26.72</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>27.48</v>
+        <v>27.29</v>
       </c>
       <c r="L8" s="1" t="n">
         <f aca="false">J8/$C8</f>
-        <v>6.7275</v>
+        <v>6.68</v>
       </c>
       <c r="M8" s="1" t="n">
         <f aca="false">K8/$C8</f>
-        <v>6.87</v>
+        <v>6.8225</v>
       </c>
       <c r="N8" s="1" t="n">
         <f aca="false">J8 / K8</f>
-        <v>0.979257641921397</v>
+        <v>0.979113228288751</v>
       </c>
       <c r="O8" s="5"/>
       <c r="P8" s="1" t="n">
         <f aca="false">G8 - L8</f>
-        <v>-0.0614999999999997</v>
+        <v>-0.0139999999999993</v>
       </c>
       <c r="Q8" s="1" t="n">
         <f aca="false">H8 - M8</f>
-        <v>-0.0679591836734694</v>
+        <v>-0.02045918367347</v>
       </c>
       <c r="R8" s="1" t="n">
         <f aca="false">$B$6 - N8</f>
-        <v>0.000742358078602567</v>
+        <v>0.000886771711249512</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -560,35 +553,35 @@
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="1" t="n">
-        <v>33.61</v>
+        <v>33.4</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>34.28</v>
+        <v>34.06</v>
       </c>
       <c r="L9" s="1" t="n">
         <f aca="false">J9/$C9</f>
-        <v>6.722</v>
+        <v>6.68</v>
       </c>
       <c r="M9" s="1" t="n">
         <f aca="false">K9/$C9</f>
-        <v>6.856</v>
+        <v>6.812</v>
       </c>
       <c r="N9" s="1" t="n">
         <f aca="false">J9 / K9</f>
-        <v>0.980455075845974</v>
+        <v>0.98062243100411</v>
       </c>
       <c r="O9" s="5"/>
       <c r="P9" s="1" t="n">
         <f aca="false">G9 - L9</f>
-        <v>-0.0560000000000001</v>
+        <v>-0.0139999999999993</v>
       </c>
       <c r="Q9" s="1" t="n">
         <f aca="false">H9 - M9</f>
-        <v>-0.0539591836734701</v>
+        <v>-0.00995918367347048</v>
       </c>
       <c r="R9" s="1" t="n">
         <f aca="false">$B$6 - N9</f>
-        <v>-0.000455075845974262</v>
+        <v>-0.000622431004110302</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -614,35 +607,35 @@
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="1" t="n">
-        <v>40.34</v>
+        <v>40.1</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>41.11</v>
+        <v>40.86</v>
       </c>
       <c r="L10" s="1" t="n">
         <f aca="false">J10/$C10</f>
-        <v>6.72333333333333</v>
+        <v>6.68333333333333</v>
       </c>
       <c r="M10" s="1" t="n">
         <f aca="false">K10/$C10</f>
-        <v>6.85166666666667</v>
+        <v>6.81</v>
       </c>
       <c r="N10" s="1" t="n">
         <f aca="false">J10 / K10</f>
-        <v>0.981269764047677</v>
+        <v>0.981399902104748</v>
       </c>
       <c r="O10" s="5"/>
       <c r="P10" s="1" t="n">
         <f aca="false">G10 - L10</f>
-        <v>-0.0573333333333332</v>
+        <v>-0.0173333333333332</v>
       </c>
       <c r="Q10" s="1" t="n">
         <f aca="false">H10 - M10</f>
-        <v>-0.049625850340135</v>
+        <v>-0.00795918367346982</v>
       </c>
       <c r="R10" s="1" t="n">
         <f aca="false">$B$6 - N10</f>
-        <v>-0.00126976404767709</v>
+        <v>-0.00139990210474794</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -668,35 +661,35 @@
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="1" t="n">
-        <v>47.09</v>
+        <v>46.82</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>47.97</v>
+        <v>47.7</v>
       </c>
       <c r="L11" s="1" t="n">
         <f aca="false">J11/$C11</f>
-        <v>6.72714285714286</v>
+        <v>6.68857142857143</v>
       </c>
       <c r="M11" s="1" t="n">
         <f aca="false">K11/$C11</f>
-        <v>6.85285714285714</v>
+        <v>6.81428571428572</v>
       </c>
       <c r="N11" s="1" t="n">
         <f aca="false">J11 / K11</f>
-        <v>0.981655201167396</v>
+        <v>0.981551362683438</v>
       </c>
       <c r="O11" s="5"/>
       <c r="P11" s="1" t="n">
         <f aca="false">G11 - L11</f>
-        <v>-0.0611428571428583</v>
+        <v>-0.0225714285714282</v>
       </c>
       <c r="Q11" s="1" t="n">
         <f aca="false">H11 - M11</f>
-        <v>-0.0508163265306116</v>
+        <v>-0.0122448979591852</v>
       </c>
       <c r="R11" s="1" t="n">
         <f aca="false">$B$6 - N11</f>
-        <v>-0.00165520116739637</v>
+        <v>-0.00155136268343814</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -722,35 +715,35 @@
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="1" t="n">
-        <v>53.87</v>
+        <v>53.56</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>54.87</v>
+        <v>54.55</v>
       </c>
       <c r="L12" s="1" t="n">
         <f aca="false">J12/$C12</f>
-        <v>6.73375</v>
+        <v>6.695</v>
       </c>
       <c r="M12" s="1" t="n">
         <f aca="false">K12/$C12</f>
-        <v>6.85875</v>
+        <v>6.81875</v>
       </c>
       <c r="N12" s="1" t="n">
         <f aca="false">J12 / K12</f>
-        <v>0.981775104793147</v>
+        <v>0.981851512373969</v>
       </c>
       <c r="O12" s="5"/>
       <c r="P12" s="1" t="n">
         <f aca="false">G12 - L12</f>
-        <v>-0.0677499999999993</v>
+        <v>-0.0289999999999999</v>
       </c>
       <c r="Q12" s="1" t="n">
         <f aca="false">H12 - M12</f>
-        <v>-0.056709183673469</v>
+        <v>-0.0167091836734699</v>
       </c>
       <c r="R12" s="1" t="n">
         <f aca="false">$B$6 - N12</f>
-        <v>-0.00177510479314746</v>
+        <v>-0.00185151237396897</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -776,35 +769,35 @@
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="1" t="n">
-        <v>60.68</v>
+        <v>60.33</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>61.8</v>
+        <v>61.44</v>
       </c>
       <c r="L13" s="1" t="n">
         <f aca="false">J13/$C13</f>
-        <v>6.74222222222222</v>
+        <v>6.70333333333333</v>
       </c>
       <c r="M13" s="1" t="n">
         <f aca="false">K13/$C13</f>
-        <v>6.86666666666667</v>
+        <v>6.82666666666667</v>
       </c>
       <c r="N13" s="1" t="n">
         <f aca="false">J13 / K13</f>
-        <v>0.981877022653722</v>
+        <v>0.98193359375</v>
       </c>
       <c r="O13" s="5"/>
       <c r="P13" s="1" t="n">
         <f aca="false">G13 - L13</f>
-        <v>-0.0762222222222215</v>
+        <v>-0.0373333333333328</v>
       </c>
       <c r="Q13" s="1" t="n">
         <f aca="false">H13 - M13</f>
-        <v>-0.0646258503401356</v>
+        <v>-0.0246258503401364</v>
       </c>
       <c r="R13" s="1" t="n">
         <f aca="false">$B$6 - N13</f>
-        <v>-0.00187702265372169</v>
+        <v>-0.00193359375000002</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -830,378 +823,92 @@
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="1" t="n">
-        <v>67.5</v>
+        <v>67.11</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>68.77</v>
+        <v>68.36</v>
       </c>
       <c r="L14" s="1" t="n">
         <f aca="false">J14/$C14</f>
-        <v>6.75</v>
+        <v>6.711</v>
       </c>
       <c r="M14" s="1" t="n">
         <f aca="false">K14/$C14</f>
-        <v>6.877</v>
+        <v>6.836</v>
       </c>
       <c r="N14" s="1" t="n">
         <f aca="false">J14 / K14</f>
-        <v>0.981532645048713</v>
+        <v>0.981714452896431</v>
       </c>
       <c r="O14" s="5"/>
       <c r="P14" s="1" t="n">
         <f aca="false">G14 - L14</f>
-        <v>-0.0840000000000005</v>
+        <v>-0.0449999999999999</v>
       </c>
       <c r="Q14" s="1" t="n">
         <f aca="false">H14 - M14</f>
-        <v>-0.07495918367347</v>
+        <v>-0.0339591836734705</v>
       </c>
       <c r="R14" s="1" t="n">
         <f aca="false">$B$6 - N14</f>
-        <v>-0.0015326450487132</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="O15" s="5"/>
+        <v>-0.00171445289643069</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="s">
+      <c r="A16" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="1" t="n">
-        <f aca="false">$B$5 *C16</f>
-        <v>73.326</v>
-      </c>
-      <c r="F16" s="1" t="n">
-        <f aca="false">E16/$B$6</f>
-        <v>74.8224489795918</v>
-      </c>
-      <c r="G16" s="1" t="n">
-        <f aca="false">E16/$C16</f>
-        <v>6.666</v>
-      </c>
-      <c r="H16" s="1" t="n">
-        <f aca="false">F16/$C16</f>
-        <v>6.80204081632653</v>
-      </c>
-      <c r="I16" s="5"/>
-      <c r="J16" s="1" t="n">
-        <v>74.36</v>
-      </c>
-      <c r="K16" s="1" t="n">
-        <v>75.76</v>
-      </c>
-      <c r="L16" s="1" t="n">
-        <f aca="false">J16/$C16</f>
-        <v>6.76</v>
-      </c>
-      <c r="M16" s="1" t="n">
-        <f aca="false">K16/$C16</f>
-        <v>6.88727272727273</v>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="O16" s="5"/>
-      <c r="P16" s="1" t="n">
-        <f aca="false">G16 - L16</f>
-        <v>-0.0939999999999994</v>
-      </c>
-      <c r="Q16" s="1" t="n">
-        <f aca="false">H16 - M16</f>
-        <v>-0.085231910946197</v>
-      </c>
-      <c r="R16" s="1" t="n">
-        <f aca="false">$B$6 - N16</f>
-        <v>-0.001</v>
+      <c r="B16" s="0" t="n">
+        <v>208</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="5" t="n">
+      <c r="A17" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="1" t="n">
-        <f aca="false">$B$5 *C17</f>
-        <v>99.99</v>
-      </c>
-      <c r="F17" s="1" t="n">
-        <f aca="false">E17/$B$6</f>
-        <v>102.030612244898</v>
-      </c>
-      <c r="G17" s="1" t="n">
-        <f aca="false">E17/$C17</f>
-        <v>6.666</v>
-      </c>
-      <c r="H17" s="1" t="n">
-        <f aca="false">F17/$C17</f>
-        <v>6.80204081632653</v>
-      </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="1" t="n">
-        <v>102.03</v>
-      </c>
-      <c r="K17" s="1" t="n">
-        <v>104.1</v>
-      </c>
-      <c r="L17" s="1" t="n">
-        <f aca="false">J17/$C17</f>
-        <v>6.802</v>
-      </c>
-      <c r="M17" s="1" t="n">
-        <f aca="false">K17/$C17</f>
-        <v>6.94</v>
-      </c>
-      <c r="N17" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="O17" s="5"/>
-      <c r="P17" s="1" t="n">
-        <f aca="false">G17 - L17</f>
-        <v>-0.136</v>
-      </c>
-      <c r="Q17" s="1" t="n">
-        <f aca="false">H17 - M17</f>
-        <v>-0.137959183673469</v>
-      </c>
-      <c r="R17" s="1" t="n">
-        <f aca="false">$B$6 - N17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="1" t="n">
-        <f aca="false">$B$5 *C18</f>
-        <v>133.32</v>
-      </c>
-      <c r="F18" s="1" t="n">
-        <f aca="false">E18/$B$6</f>
-        <v>136.040816326531</v>
-      </c>
-      <c r="G18" s="1" t="n">
-        <f aca="false">E18/$C18</f>
-        <v>6.666</v>
-      </c>
-      <c r="H18" s="1" t="n">
-        <f aca="false">F18/$C18</f>
-        <v>6.80204081632653</v>
-      </c>
-      <c r="I18" s="5"/>
-      <c r="J18" s="1" t="n">
-        <v>137.18</v>
-      </c>
-      <c r="K18" s="1" t="n">
-        <v>140.29</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <f aca="false">J18/$C18</f>
-        <v>6.859</v>
-      </c>
-      <c r="M18" s="1" t="n">
-        <f aca="false">K18/$C18</f>
-        <v>7.0145</v>
-      </c>
-      <c r="N18" s="1" t="n">
-        <v>0.978</v>
-      </c>
-      <c r="O18" s="5"/>
-      <c r="P18" s="1" t="n">
-        <f aca="false">G18 - L18</f>
-        <v>-0.193000000000001</v>
-      </c>
-      <c r="Q18" s="1" t="n">
-        <f aca="false">H18 - M18</f>
-        <v>-0.21245918367347</v>
-      </c>
-      <c r="R18" s="1" t="n">
-        <f aca="false">$B$6 - N18</f>
-        <v>0.002</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="1" t="n">
-        <f aca="false">$B$5 *C19</f>
-        <v>199.98</v>
-      </c>
-      <c r="F19" s="1" t="n">
-        <f aca="false">E19/$B$6</f>
-        <v>204.061224489796</v>
-      </c>
-      <c r="G19" s="1" t="n">
-        <f aca="false">E19/$C19</f>
-        <v>6.666</v>
-      </c>
-      <c r="H19" s="1" t="n">
-        <f aca="false">F19/$C19</f>
-        <v>6.80204081632653</v>
-      </c>
-      <c r="I19" s="5"/>
-      <c r="J19" s="1" t="n">
-        <v>209.37</v>
-      </c>
-      <c r="K19" s="1" t="n">
-        <v>215.33</v>
-      </c>
-      <c r="L19" s="1" t="n">
-        <f aca="false">J19/$C19</f>
-        <v>6.979</v>
-      </c>
-      <c r="M19" s="1" t="n">
-        <f aca="false">K19/$C19</f>
-        <v>7.17766666666667</v>
-      </c>
-      <c r="N19" s="1" t="n">
-        <v>0.972</v>
-      </c>
-      <c r="O19" s="5"/>
-      <c r="P19" s="1" t="n">
-        <f aca="false">G19 - L19</f>
-        <v>-0.313</v>
-      </c>
-      <c r="Q19" s="1" t="n">
-        <f aca="false">H19 - M19</f>
-        <v>-0.375625850340136</v>
-      </c>
-      <c r="R19" s="1" t="n">
-        <f aca="false">$B$6 - N19</f>
-        <v>0.00800000000000001</v>
+      <c r="B19" s="0" t="n">
+        <v>0.99</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="1" t="n">
-        <f aca="false">$B$5 *C20</f>
-        <v>333.3</v>
-      </c>
-      <c r="F20" s="1" t="n">
-        <f aca="false">E20/$B$6</f>
-        <v>340.102040816327</v>
-      </c>
-      <c r="G20" s="1" t="n">
-        <f aca="false">E20/$C20</f>
-        <v>6.666</v>
-      </c>
-      <c r="H20" s="1" t="n">
-        <f aca="false">F20/$C20</f>
-        <v>6.80204081632653</v>
-      </c>
-      <c r="I20" s="5"/>
-      <c r="J20" s="1" t="n">
-        <v>361.33</v>
-      </c>
-      <c r="K20" s="1" t="n">
-        <v>376.59</v>
-      </c>
-      <c r="L20" s="1" t="n">
-        <f aca="false">J20/$C20</f>
-        <v>7.2266</v>
-      </c>
-      <c r="M20" s="1" t="n">
-        <f aca="false">K20/$C20</f>
-        <v>7.5318</v>
-      </c>
-      <c r="N20" s="1" t="n">
-        <v>0.959</v>
-      </c>
-      <c r="O20" s="5"/>
-      <c r="P20" s="1" t="n">
-        <f aca="false">G20 - L20</f>
-        <v>-0.560599999999999</v>
-      </c>
-      <c r="Q20" s="1" t="n">
-        <f aca="false">H20 - M20</f>
-        <v>-0.729759183673468</v>
-      </c>
-      <c r="R20" s="1" t="n">
-        <f aca="false">$B$6 - N20</f>
-        <v>0.021</v>
+      <c r="A20" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <f aca="false">BREAKER_RATING_A * CONTINUOUS_DUTY_DERATE</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="0" t="n">
+        <f aca="false">PANEL_VOLTAGE_V * ev_pilot_current_a / 1000</f>
+        <v>6.656</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B22" s="0" t="n">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" s="0" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="0" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="0" t="n">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="0" t="n">
-        <f aca="false">BREAKER_RATING_A * CONTINUOUS_DUTY_DERATE</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" s="0" t="n">
-        <f aca="false">PANEL_VOLTAGE_V * ev_pilot_current_a / 1000</f>
-        <v>6.656</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" s="0" t="n">
         <f aca="false">ev_apparent_power_kva * EV_TRUE_POWER_FACTOR</f>
         <v>6.58944</v>
       </c>

</xml_diff>

<commit_message>
Updated docs/session/Rough_kW_kVA_Table.xlsx with values with 3 decimal digits.
</commit_message>
<xml_diff>
--- a/docs/session/Rough_kW_kVA_Table.xlsx
+++ b/docs/session/Rough_kW_kVA_Table.xlsx
@@ -224,7 +224,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="1.68"/>
@@ -331,35 +331,35 @@
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="1" t="n">
-        <v>6.8</v>
+        <v>6.797</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>7.22</v>
+        <v>7.218</v>
       </c>
       <c r="L5" s="1" t="n">
         <f aca="false">J5/$C5</f>
-        <v>6.8</v>
+        <v>6.797</v>
       </c>
       <c r="M5" s="1" t="n">
         <f aca="false">K5/$C5</f>
-        <v>7.22</v>
+        <v>7.218</v>
       </c>
       <c r="N5" s="1" t="n">
         <f aca="false">J5 / K5</f>
-        <v>0.941828254847645</v>
+        <v>0.941673593793295</v>
       </c>
       <c r="O5" s="5"/>
       <c r="P5" s="1" t="n">
         <f aca="false">G5 - L5</f>
-        <v>-0.133999999999999</v>
+        <v>-0.130999999999999</v>
       </c>
       <c r="Q5" s="1" t="n">
         <f aca="false">H5 - M5</f>
-        <v>-0.41795918367347</v>
+        <v>-0.41595918367347</v>
       </c>
       <c r="R5" s="1" t="n">
         <f aca="false">$B$6 - N5</f>
-        <v>0.0381717451523546</v>
+        <v>0.0383264062067055</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -391,35 +391,35 @@
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="1" t="n">
-        <v>13.42</v>
+        <v>13.417</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>13.85</v>
+        <v>13.846</v>
       </c>
       <c r="L6" s="1" t="n">
         <f aca="false">J6/$C6</f>
-        <v>6.71</v>
+        <v>6.7085</v>
       </c>
       <c r="M6" s="1" t="n">
         <f aca="false">K6/$C6</f>
-        <v>6.925</v>
+        <v>6.923</v>
       </c>
       <c r="N6" s="1" t="n">
         <f aca="false">J6 / K6</f>
-        <v>0.968953068592058</v>
+        <v>0.969016322403582</v>
       </c>
       <c r="O6" s="5"/>
       <c r="P6" s="1" t="n">
         <f aca="false">G6 - L6</f>
-        <v>-0.0439999999999996</v>
+        <v>-0.0424999999999995</v>
       </c>
       <c r="Q6" s="1" t="n">
         <f aca="false">H6 - M6</f>
-        <v>-0.12295918367347</v>
+        <v>-0.12095918367347</v>
       </c>
       <c r="R6" s="1" t="n">
         <f aca="false">$B$6 - N6</f>
-        <v>0.0110469314079422</v>
+        <v>0.0109836775964177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -445,35 +445,35 @@
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="1" t="n">
-        <v>20.06</v>
+        <v>20.057</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>20.55</v>
+        <v>20.548</v>
       </c>
       <c r="L7" s="1" t="n">
         <f aca="false">J7/$C7</f>
-        <v>6.68666666666667</v>
+        <v>6.68566666666667</v>
       </c>
       <c r="M7" s="1" t="n">
         <f aca="false">K7/$C7</f>
-        <v>6.85</v>
+        <v>6.84933333333333</v>
       </c>
       <c r="N7" s="1" t="n">
         <f aca="false">J7 / K7</f>
-        <v>0.976155717761557</v>
+        <v>0.976104730387386</v>
       </c>
       <c r="O7" s="5"/>
       <c r="P7" s="1" t="n">
         <f aca="false">G7 - L7</f>
-        <v>-0.0206666666666662</v>
+        <v>-0.0196666666666658</v>
       </c>
       <c r="Q7" s="1" t="n">
         <f aca="false">H7 - M7</f>
-        <v>-0.0479591836734707</v>
+        <v>-0.0472925170068033</v>
       </c>
       <c r="R7" s="1" t="n">
         <f aca="false">$B$6 - N7</f>
-        <v>0.00384428223844291</v>
+        <v>0.00389526961261433</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -499,35 +499,35 @@
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="1" t="n">
-        <v>26.72</v>
+        <v>26.718</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>27.29</v>
+        <v>27.289</v>
       </c>
       <c r="L8" s="1" t="n">
         <f aca="false">J8/$C8</f>
-        <v>6.68</v>
+        <v>6.6795</v>
       </c>
       <c r="M8" s="1" t="n">
         <f aca="false">K8/$C8</f>
-        <v>6.8225</v>
+        <v>6.82225</v>
       </c>
       <c r="N8" s="1" t="n">
         <f aca="false">J8 / K8</f>
-        <v>0.979113228288751</v>
+        <v>0.979075818095203</v>
       </c>
       <c r="O8" s="5"/>
       <c r="P8" s="1" t="n">
         <f aca="false">G8 - L8</f>
-        <v>-0.0139999999999993</v>
+        <v>-0.0134999999999996</v>
       </c>
       <c r="Q8" s="1" t="n">
         <f aca="false">H8 - M8</f>
-        <v>-0.02045918367347</v>
+        <v>-0.0202091836734706</v>
       </c>
       <c r="R8" s="1" t="n">
         <f aca="false">$B$6 - N8</f>
-        <v>0.000886771711249512</v>
+        <v>0.000924181904796817</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -553,35 +553,35 @@
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="1" t="n">
-        <v>33.4</v>
+        <v>33.399</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>34.06</v>
+        <v>34.061</v>
       </c>
       <c r="L9" s="1" t="n">
         <f aca="false">J9/$C9</f>
-        <v>6.68</v>
+        <v>6.6798</v>
       </c>
       <c r="M9" s="1" t="n">
         <f aca="false">K9/$C9</f>
-        <v>6.812</v>
+        <v>6.8122</v>
       </c>
       <c r="N9" s="1" t="n">
         <f aca="false">J9 / K9</f>
-        <v>0.98062243100411</v>
+        <v>0.980564281729838</v>
       </c>
       <c r="O9" s="5"/>
       <c r="P9" s="1" t="n">
         <f aca="false">G9 - L9</f>
-        <v>-0.0139999999999993</v>
+        <v>-0.0137999999999998</v>
       </c>
       <c r="Q9" s="1" t="n">
         <f aca="false">H9 - M9</f>
-        <v>-0.00995918367347048</v>
+        <v>-0.01015918367347</v>
       </c>
       <c r="R9" s="1" t="n">
         <f aca="false">$B$6 - N9</f>
-        <v>-0.000622431004110302</v>
+        <v>-0.00056428172983769</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -610,7 +610,7 @@
         <v>40.1</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>40.86</v>
+        <v>40.864</v>
       </c>
       <c r="L10" s="1" t="n">
         <f aca="false">J10/$C10</f>
@@ -618,11 +618,11 @@
       </c>
       <c r="M10" s="1" t="n">
         <f aca="false">K10/$C10</f>
-        <v>6.81</v>
+        <v>6.81066666666667</v>
       </c>
       <c r="N10" s="1" t="n">
         <f aca="false">J10 / K10</f>
-        <v>0.981399902104748</v>
+        <v>0.981303837118246</v>
       </c>
       <c r="O10" s="5"/>
       <c r="P10" s="1" t="n">
@@ -631,11 +631,11 @@
       </c>
       <c r="Q10" s="1" t="n">
         <f aca="false">H10 - M10</f>
-        <v>-0.00795918367346982</v>
+        <v>-0.00862585034013641</v>
       </c>
       <c r="R10" s="1" t="n">
         <f aca="false">$B$6 - N10</f>
-        <v>-0.00139990210474794</v>
+        <v>-0.001303837118246</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -661,35 +661,35 @@
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="1" t="n">
-        <v>46.82</v>
+        <v>46.822</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>47.7</v>
+        <v>47.695</v>
       </c>
       <c r="L11" s="1" t="n">
         <f aca="false">J11/$C11</f>
-        <v>6.68857142857143</v>
+        <v>6.68885714285714</v>
       </c>
       <c r="M11" s="1" t="n">
         <f aca="false">K11/$C11</f>
-        <v>6.81428571428572</v>
+        <v>6.81357142857143</v>
       </c>
       <c r="N11" s="1" t="n">
         <f aca="false">J11 / K11</f>
-        <v>0.981551362683438</v>
+        <v>0.981696194569661</v>
       </c>
       <c r="O11" s="5"/>
       <c r="P11" s="1" t="n">
         <f aca="false">G11 - L11</f>
-        <v>-0.0225714285714282</v>
+        <v>-0.0228571428571431</v>
       </c>
       <c r="Q11" s="1" t="n">
         <f aca="false">H11 - M11</f>
-        <v>-0.0122448979591852</v>
+        <v>-0.0115306122448988</v>
       </c>
       <c r="R11" s="1" t="n">
         <f aca="false">$B$6 - N11</f>
-        <v>-0.00155136268343814</v>
+        <v>-0.00169619456966141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -715,35 +715,35 @@
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="1" t="n">
-        <v>53.56</v>
+        <v>53.564</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>54.55</v>
+        <v>54.555</v>
       </c>
       <c r="L12" s="1" t="n">
         <f aca="false">J12/$C12</f>
-        <v>6.695</v>
+        <v>6.6955</v>
       </c>
       <c r="M12" s="1" t="n">
         <f aca="false">K12/$C12</f>
-        <v>6.81875</v>
+        <v>6.819375</v>
       </c>
       <c r="N12" s="1" t="n">
         <f aca="false">J12 / K12</f>
-        <v>0.981851512373969</v>
+        <v>0.981834845568692</v>
       </c>
       <c r="O12" s="5"/>
       <c r="P12" s="1" t="n">
         <f aca="false">G12 - L12</f>
-        <v>-0.0289999999999999</v>
+        <v>-0.0294999999999996</v>
       </c>
       <c r="Q12" s="1" t="n">
         <f aca="false">H12 - M12</f>
-        <v>-0.0167091836734699</v>
+        <v>-0.0173341836734702</v>
       </c>
       <c r="R12" s="1" t="n">
         <f aca="false">$B$6 - N12</f>
-        <v>-0.00185151237396897</v>
+        <v>-0.00183484556869218</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -769,35 +769,35 @@
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="1" t="n">
-        <v>60.33</v>
+        <v>60.327</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>61.44</v>
+        <v>61.443</v>
       </c>
       <c r="L13" s="1" t="n">
         <f aca="false">J13/$C13</f>
-        <v>6.70333333333333</v>
+        <v>6.703</v>
       </c>
       <c r="M13" s="1" t="n">
         <f aca="false">K13/$C13</f>
-        <v>6.82666666666667</v>
+        <v>6.827</v>
       </c>
       <c r="N13" s="1" t="n">
         <f aca="false">J13 / K13</f>
-        <v>0.98193359375</v>
+        <v>0.98183682437381</v>
       </c>
       <c r="O13" s="5"/>
       <c r="P13" s="1" t="n">
         <f aca="false">G13 - L13</f>
-        <v>-0.0373333333333328</v>
+        <v>-0.036999999999999</v>
       </c>
       <c r="Q13" s="1" t="n">
         <f aca="false">H13 - M13</f>
-        <v>-0.0246258503401364</v>
+        <v>-0.0249591836734702</v>
       </c>
       <c r="R13" s="1" t="n">
         <f aca="false">$B$6 - N13</f>
-        <v>-0.00193359375000002</v>
+        <v>-0.00183682437380994</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -826,7 +826,7 @@
         <v>67.11</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>68.36</v>
+        <v>68.359</v>
       </c>
       <c r="L14" s="1" t="n">
         <f aca="false">J14/$C14</f>
@@ -834,11 +834,11 @@
       </c>
       <c r="M14" s="1" t="n">
         <f aca="false">K14/$C14</f>
-        <v>6.836</v>
+        <v>6.8359</v>
       </c>
       <c r="N14" s="1" t="n">
         <f aca="false">J14 / K14</f>
-        <v>0.981714452896431</v>
+        <v>0.981728814055209</v>
       </c>
       <c r="O14" s="5"/>
       <c r="P14" s="1" t="n">
@@ -847,11 +847,11 @@
       </c>
       <c r="Q14" s="1" t="n">
         <f aca="false">H14 - M14</f>
-        <v>-0.0339591836734705</v>
+        <v>-0.0338591836734698</v>
       </c>
       <c r="R14" s="1" t="n">
         <f aca="false">$B$6 - N14</f>
-        <v>-0.00171445289643069</v>
+        <v>-0.00172881405520864</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>